<commit_message>
Itemizado Grupo 7: columnas de valorizacion, hoja de insumos y hoja de gastos generales
</commit_message>
<xml_diff>
--- a/Trabajo/01_Itemizado_Grupo7.xlsx
+++ b/Trabajo/01_Itemizado_Grupo7.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itemizado Grupo 7" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insumos y Rendimientos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gastos Generales" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +38,12 @@
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,8 +65,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -82,11 +98,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,6 +156,23 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -470,6 +547,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,16 +582,32 @@
           <t>PU DETALLADO</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PU REF. ($/unidad)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>MONTO ($)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>1.0  MOVIMIENTO DE TIERRAS, FUNDACIONES Y VIALIDAD</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="19" t="n"/>
+      <c r="H2" s="19" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -537,6 +632,11 @@
         <v>466</v>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9">
+        <f>IF(G3="","",E3*G3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -561,6 +661,11 @@
         <v>20354</v>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9">
+        <f>IF(G4="","",E4*G4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -585,6 +690,11 @@
         <v>7740</v>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9">
+        <f>IF(G5="","",E5*G5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -609,6 +719,11 @@
         <v>2944</v>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9">
+        <f>IF(G6="","",E6*G6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -633,6 +748,11 @@
         <v>2198</v>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9">
+        <f>IF(G7="","",E7*G7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -657,6 +777,11 @@
         <v>3299</v>
       </c>
       <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9">
+        <f>IF(G8="","",E8*G8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -681,6 +806,11 @@
         <v>3398</v>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9">
+        <f>IF(G9="","",E9*G9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -705,6 +835,11 @@
         <v>1955</v>
       </c>
       <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9">
+        <f>IF(G10="","",E10*G10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -729,6 +864,11 @@
         <v>1699</v>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9">
+        <f>IF(G11="","",E11*G11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -753,6 +893,11 @@
         <v>16024</v>
       </c>
       <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9">
+        <f>IF(G12="","",E12*G12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -777,6 +922,11 @@
         <v>9756</v>
       </c>
       <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9">
+        <f>IF(G13="","",E13*G13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -801,6 +951,11 @@
         <v>1965</v>
       </c>
       <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9">
+        <f>IF(G14="","",E14*G14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -825,6 +980,11 @@
         <v>3204</v>
       </c>
       <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9">
+        <f>IF(G15="","",E15*G15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -853,6 +1013,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9">
+        <f>IF(G16="","",E16*G16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -877,6 +1042,11 @@
         <v>1758</v>
       </c>
       <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9">
+        <f>IF(G17="","",E17*G17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -901,6 +1071,11 @@
         <v>891</v>
       </c>
       <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9">
+        <f>IF(G18="","",E18*G18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -925,6 +1100,11 @@
         <v>62</v>
       </c>
       <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9">
+        <f>IF(G19="","",E19*G19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -949,6 +1129,11 @@
         <v>121</v>
       </c>
       <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9">
+        <f>IF(G20="","",E20*G20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -977,6 +1162,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9">
+        <f>IF(G21="","",E21*G21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1001,6 +1191,11 @@
         <v>430</v>
       </c>
       <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9">
+        <f>IF(G22="","",E22*G22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1025,6 +1220,11 @@
         <v>42496</v>
       </c>
       <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9">
+        <f>IF(G23="","",E23*G23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1049,6 +1249,11 @@
         <v>10277</v>
       </c>
       <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9">
+        <f>IF(G24="","",E24*G24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1073,6 +1278,11 @@
         <v>21028</v>
       </c>
       <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9">
+        <f>IF(G25="","",E25*G25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1097,6 +1307,11 @@
         <v>23885</v>
       </c>
       <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9">
+        <f>IF(G26="","",E26*G26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1121,6 +1336,11 @@
         <v>60</v>
       </c>
       <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9">
+        <f>IF(G27="","",E27*G27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1149,6 +1369,11 @@
           <t>X</t>
         </is>
       </c>
+      <c r="G28" s="9" t="n"/>
+      <c r="H28" s="9">
+        <f>IF(G28="","",E28*G28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1173,16 +1398,27 @@
         <v>1359</v>
       </c>
       <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9">
+        <f>IF(G29="","",E29*G29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>2.0  ESTRUCTURAS, REVESTIMIENTOS, CUBIERTAS Y TERMINACIONES</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1207,6 +1443,11 @@
         <v>581078</v>
       </c>
       <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9">
+        <f>IF(G31="","",E31*G31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1231,6 +1472,11 @@
         <v>15319</v>
       </c>
       <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9">
+        <f>IF(G32="","",E32*G32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1255,6 +1501,11 @@
         <v>7626</v>
       </c>
       <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9">
+        <f>IF(G33="","",E33*G33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1279,6 +1530,11 @@
         <v>2211</v>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9">
+        <f>IF(G34="","",E34*G34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1303,6 +1559,11 @@
         <v>581</v>
       </c>
       <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9">
+        <f>IF(G35="","",E35*G35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1327,6 +1588,11 @@
         <v>32</v>
       </c>
       <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9">
+        <f>IF(G36="","",E36*G36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1351,6 +1617,11 @@
         <v>32</v>
       </c>
       <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9">
+        <f>IF(G37="","",E37*G37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1375,6 +1646,11 @@
         <v>781</v>
       </c>
       <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="9">
+        <f>IF(G38="","",E38*G38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1399,6 +1675,11 @@
         <v>58</v>
       </c>
       <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9">
+        <f>IF(G39="","",E39*G39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -1423,6 +1704,11 @@
         <v>35</v>
       </c>
       <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9">
+        <f>IF(G40="","",E40*G40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1447,6 +1733,11 @@
         <v>22</v>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9">
+        <f>IF(G41="","",E41*G41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -1471,6 +1762,11 @@
         <v>24</v>
       </c>
       <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9">
+        <f>IF(G42="","",E42*G42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1495,6 +1791,11 @@
         <v>238</v>
       </c>
       <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9">
+        <f>IF(G43="","",E43*G43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -1523,24 +1824,369 @@
           <t>X</t>
         </is>
       </c>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9">
+        <f>IF(G44="","",E44*G44)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" s="6" t="inlineStr">
         <is>
           <t>TOTAL GRUPO 7 (solo partidas con cantidad)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>RESUMEN DE VALORIZACIÓN (GRUPO 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Costo directo total ($)</t>
+        </is>
+      </c>
+      <c r="C49" s="12">
+        <f>SUM(H3:H44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Gastos generales (%)</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Gastos generales ($)</t>
+        </is>
+      </c>
+      <c r="C51" s="12">
+        <f>C49*C50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad (%)</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad ($)</t>
+        </is>
+      </c>
+      <c r="C53" s="12">
+        <f>(C49+C51)*C52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>PRECIO DE VENTA TOTAL ($)</t>
+        </is>
+      </c>
+      <c r="C54" s="15">
+        <f>C49+C51+C53</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ítem partida</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Insumo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cantidad por unidad de partida</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Precio unitario ($)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ítem de gasto general (enunciado)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Valor estimado ($)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fuente / justificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Personal administrativo y directivo del contrato (residente, jefe de terreno, jefe administrativo, prevencionista de riesgos, topógrafo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Personal auxiliar (ayudante de topografía, bodeguero, personal de casino, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Equipamiento de topografía</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Laboratorio, estudios de suelo y estructural</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Insumos de instalaciones (agua, gas, electricidad, agua potable, internet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fotografías, videos, planos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Movilización</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Combustible</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Viáticos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Traslado de maquinarias</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Gastos de representación y oficina central</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Boleta de garantía</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Seguro de todo riesgo montaje y construcción</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Letrero de obras</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Libro de obra digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Limpieza de obra diaria y final</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS GENERALES ($)</t>
+        </is>
+      </c>
+      <c r="C18" s="16">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>% sobre costo directo</t>
+        </is>
+      </c>
+      <c r="C19" s="17">
+        <f>'Itemizado Grupo 7'!C50</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>